<commit_message>
feat: add user signup and public access controls
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -244,22 +244,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Access</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Owner is logged in</t>
+          <t>App is running</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Open Access dialog</t>
+          <t>Open create-user mode from login screen and submit valid data</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>All users and current roles are visible</t>
+          <t>New user is created, signed in and shown in the top bar</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -269,7 +269,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -296,12 +296,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Grant viewer role to viewer user</t>
+          <t>Right-click data room and open Manage access</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Viewer can see the data room in their list</t>
+          <t>Access dialog opens from the context menu</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -311,7 +311,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -333,17 +333,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Viewer is logged in</t>
+          <t>Owner is logged in</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Open shared data room</t>
+          <t>Search Val in the access dialog</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Viewer can browse and preview files</t>
+          <t>Only matching users are shown</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -353,7 +353,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -375,17 +375,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Viewer is logged in</t>
+          <t>Owner is logged in</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Try to create folder or upload PDF</t>
+          <t>Set Available to everyone to viewer</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Write controls are disabled or API returns forbidden</t>
+          <t>Right panel shows Everyone with VIEWER role</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -417,17 +417,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Owner is logged in</t>
+          <t>Public viewer access is enabled</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Grant editor role to editor user</t>
+          <t>Create a new user and open data room list</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Editor can create, rename, move and delete files/folders</t>
+          <t>New user can see the public data room as VIEWER</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -464,12 +464,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Try to remove owner access</t>
+          <t>Grant viewer role to viewer user</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>System rejects owner access change</t>
+          <t>Viewer can see the data room in their list</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -496,22 +496,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Data rooms</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Owner is logged in</t>
+          <t>Viewer is logged in</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Create a new data room</t>
+          <t>Open shared data room</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>New data room appears in sidebar with OWNER role</t>
+          <t>Viewer can browse and preview files</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -538,27 +538,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Data rooms</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Owner is logged in</t>
+          <t>Viewer is logged in</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rename data room</t>
+          <t>Try to create folder or upload PDF</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>New name is shown in sidebar and header</t>
+          <t>Write controls are disabled or API returns forbidden</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data rooms</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -590,12 +590,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Delete data room</t>
+          <t>Grant editor role to editor user</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Data room, items, access records and blobs are removed</t>
+          <t>Editor can create, rename, move and delete files/folders</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -622,22 +622,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Folders</t>
+          <t>Access</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Editable data room is selected</t>
+          <t>Owner is logged in</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Create folder in root</t>
+          <t>Try to remove owner access</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Folder appears in the table</t>
+          <t>System rejects owner access change</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -664,22 +664,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Folders</t>
+          <t>Data rooms</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Folder exists</t>
+          <t>Owner is logged in</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Open folder and create nested folder</t>
+          <t>Create a new data room</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Nested folder is created under parent</t>
+          <t>New data room appears in sidebar with OWNER role</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -706,22 +706,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Folders</t>
+          <t>Data rooms</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Nested folder is open</t>
+          <t>Owner is logged in</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Use breadcrumb to return to root</t>
+          <t>Rename data room</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Root folder contents are displayed</t>
+          <t>New name is shown in sidebar and header</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -748,27 +748,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Folders</t>
+          <t>Data rooms</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Folder exists</t>
+          <t>Owner is logged in</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Rename folder</t>
+          <t>Delete data room</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Folder row shows new name</t>
+          <t>Data room, items, access records and blobs are removed</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Folder has nested files and folders</t>
+          <t>Editable data room is selected</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Delete top-level folder</t>
+          <t>Create folder in root</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>All descendants and file blobs are deleted</t>
+          <t>Folder appears in the table</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -832,22 +832,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Files</t>
+          <t>Folders</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Editable data room is selected</t>
+          <t>Folder exists</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Upload a valid PDF</t>
+          <t>Open folder and create nested folder</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PDF row appears and blob is stored</t>
+          <t>Nested folder is created under parent</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -874,27 +874,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Files</t>
+          <t>Folders</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Editable data room is selected</t>
+          <t>Nested folder is open</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Upload non-PDF file</t>
+          <t>Use breadcrumb to return to root</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Upload is rejected</t>
+          <t>Root folder contents are displayed</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -916,22 +916,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Files</t>
+          <t>Folders</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Report.pdf already exists</t>
+          <t>Folder exists</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Upload another Report.pdf</t>
+          <t>Rename folder</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Second file receives safe duplicate name</t>
+          <t>Folder row shows new name</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -958,22 +958,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Files</t>
+          <t>Folders</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PDF exists</t>
+          <t>Folder has nested files and folders</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Select PDF row</t>
+          <t>Delete top-level folder</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Right details panel shows metadata and preview</t>
+          <t>All descendants and file blobs are deleted</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1005,22 +1005,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PDF exists</t>
+          <t>Editable data room is selected</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Rename PDF</t>
+          <t>Upload a valid PDF</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>File row and details panel show new name</t>
+          <t>PDF row appears and blob is stored</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1047,17 +1047,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PDF exists</t>
+          <t>Editable data room is selected</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Delete PDF</t>
+          <t>Upload Dmytro_Kiselov_Full-Stack_Developer.pdf from test-assets/resumes</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>File row disappears and blob content is unavailable</t>
+          <t>Resume PDF row appears and opens in preview</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1084,22 +1084,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Move</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Two folders exist</t>
+          <t>Editable data room is selected</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Move file from root into folder</t>
+          <t>Upload every PDF from test-assets/resumes</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>File is shown inside target folder only</t>
+          <t>All resume versions upload successfully</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1126,22 +1126,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Move</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nested folders exist</t>
+          <t>Editable data room is selected</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Move folder into another folder</t>
+          <t>Upload non-PDF file</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Folder path updates and breadcrumb works</t>
+          <t>Upload is rejected</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1168,27 +1168,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Move</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Parent and child folders exist</t>
+          <t>Report.pdf already exists</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Try to move parent into child</t>
+          <t>Upload another Report.pdf</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>System rejects invalid move</t>
+          <t>Second file receives safe duplicate name</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1210,22 +1210,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PDF with text content is uploaded</t>
+          <t>PDF exists</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Search by visible file name</t>
+          <t>Select PDF row</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Matching file is shown</t>
+          <t>Right details panel shows metadata and preview</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1252,27 +1252,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PDF with indexed text is uploaded</t>
+          <t>PDF exists</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Search by a word inside PDF content</t>
+          <t>Rename PDF</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Matching file is shown</t>
+          <t>File row and details panel show new name</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1294,32 +1294,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Files</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Files/folders exist</t>
+          <t>PDF exists</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Search for missing term</t>
+          <t>Delete PDF</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Empty state is shown</t>
+          <t>File row disappears and blob content is unavailable</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Automated</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1336,22 +1336,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Viewer</t>
+          <t>Move</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PDF is selected</t>
+          <t>Two folders exist</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Click Open in data room viewer</t>
+          <t>Move file from root into folder</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Fullscreen modal opens inside app UI</t>
+          <t>File is shown inside target folder only</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1378,27 +1378,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Viewer</t>
+          <t>Move</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fullscreen viewer is open</t>
+          <t>Nested folders exist</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Close viewer</t>
+          <t>Move folder into another folder</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>User returns to workspace without navigation loss</t>
+          <t>Folder path updates and breadcrumb works</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1420,22 +1420,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>Move</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Docker stack is running</t>
+          <t>Parent and child folders exist</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Restart app container</t>
+          <t>Try to move parent into child</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Data rooms, access and item metadata remain in PostgreSQL</t>
+          <t>System rejects invalid move</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1462,22 +1462,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Blob storage</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PDF was uploaded</t>
+          <t>PDF with text content is uploaded</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Restart app container</t>
+          <t>Search by visible file name</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>PDF content remains available from upload volume</t>
+          <t>Matching file is shown</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>Automated</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1504,22 +1504,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Docker</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Docker Desktop is running</t>
+          <t>PDF with indexed text is uploaded</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Run docker compose up -d --build</t>
+          <t>Search by a word inside PDF content</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Postgres and app start with one command</t>
+          <t>Matching file is shown</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1546,41 +1546,293 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Files/folders exist</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Search for missing term</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Empty state is shown</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Viewer</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PDF is selected</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Click Open in data room viewer</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Fullscreen modal opens inside app UI</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TC-037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Viewer</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Fullscreen viewer is open</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Close viewer</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>User returns to workspace without navigation loss</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TC-038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Docker stack is running</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Restart app container</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Data rooms, access and item metadata remain in PostgreSQL</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TC-039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Blob storage</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PDF was uploaded</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Restart app container</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PDF content remains available from upload volume</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TC-040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Docker</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Docker Desktop is running</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Run docker compose up -d --build</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Postgres and app start with one command</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>TC-041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>CI</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Feature branch is pushed</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Open GitHub Actions</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Lint, typecheck, tests and build pass</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>Ready</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H36"/>
+  <autoFilter ref="A1:H42"/>
 </worksheet>
 </file>
</xml_diff>